<commit_message>
Start with empty database by default, add empty state prompt with upload/template/demo actions, and add Clear DB and persistence
</commit_message>
<xml_diff>
--- a/data/SpectraPanel_Database_Populated.xlsx
+++ b/data/SpectraPanel_Database_Populated.xlsx
@@ -1706,12 +1706,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="53" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
@@ -1764,7 +1764,7 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Rabbit</t>
+          <t>Goat</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -1774,45 +1774,37 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Alexa Fluor 488</t>
+          <t>HRP (Donkey, Invitrogen A15999)</t>
         </is>
       </c>
       <c r="D2" s="6" t="inlineStr">
         <is>
-          <t>Fluorophore</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>Green</t>
-        </is>
-      </c>
-      <c r="F2" s="6" t="n">
-        <v>490</v>
-      </c>
-      <c r="G2" s="6" t="n">
-        <v>525</v>
-      </c>
+          <t>HRP</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr"/>
+      <c r="F2" s="6" t="inlineStr"/>
+      <c r="G2" s="6" t="inlineStr"/>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>ICC, IHC, WB</t>
+          <t>WB</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Rabbit</t>
+          <t>Mouse</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>IgG (H+L)</t>
+          <t>IgM</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Alexa Fluor 555</t>
+          <t>Alexa Fluor 488 (Goat, Invitrogen A21042)</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
@@ -1822,14 +1814,14 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>Green</t>
         </is>
       </c>
       <c r="F3" s="6" t="n">
-        <v>555</v>
+        <v>490</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>565</v>
+        <v>525</v>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
@@ -1850,7 +1842,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Alexa Fluor 647</t>
+          <t>Alexa Fluor 488 (Donkey, Invitrogen A21206)</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
@@ -1860,14 +1852,14 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Far-Red</t>
+          <t>Green</t>
         </is>
       </c>
       <c r="F4" s="6" t="n">
-        <v>650</v>
+        <v>490</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>665</v>
+        <v>525</v>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
@@ -1878,37 +1870,45 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Rabbit</t>
+          <t>Chicken</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>IgG (H+L)</t>
+          <t>IgY (H+L)</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>HRP</t>
+          <t>Alexa Fluor 633 (Goat, Invitrogen A21103)</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>HRP</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="G5" s="6" t="inlineStr"/>
+          <t>Fluorophore</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Far-Red</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>632</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>647</v>
+      </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>WB</t>
+          <t>ICC, IHC, WB</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Mouse</t>
+          <t>Rabbit</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1918,7 +1918,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Alexa Fluor 488</t>
+          <t>Alexa Fluor 647 (Goat, Invitrogen A21245)</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
@@ -1928,14 +1928,14 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Green</t>
+          <t>Far-Red</t>
         </is>
       </c>
       <c r="F6" s="6" t="n">
-        <v>490</v>
+        <v>650</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>525</v>
+        <v>665</v>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
@@ -1956,7 +1956,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Alexa Fluor 555</t>
+          <t>Alexa Fluor 647 (Goat, Invitrogen A21235)</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -1966,14 +1966,14 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Red</t>
+          <t>Far-Red</t>
         </is>
       </c>
       <c r="F7" s="6" t="n">
-        <v>555</v>
+        <v>650</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>565</v>
+        <v>665</v>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
@@ -1994,7 +1994,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Alexa Fluor 647</t>
+          <t>Alexa Fluor 488 (Goat, Invitrogen A11001)</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -2004,14 +2004,14 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Far-Red</t>
+          <t>Green</t>
         </is>
       </c>
       <c r="F8" s="6" t="n">
-        <v>650</v>
+        <v>490</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>665</v>
+        <v>525</v>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
@@ -2022,7 +2022,7 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>Mouse</t>
+          <t>Rabbit</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -2032,20 +2032,28 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>HRP</t>
+          <t>Alexa Fluor Plus 647 (Goat, Invitrogen A32733)</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>HRP</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr"/>
-      <c r="F9" s="6" t="inlineStr"/>
-      <c r="G9" s="6" t="inlineStr"/>
+          <t>Fluorophore</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Far-Red</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>650</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>665</v>
+      </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>WB</t>
+          <t>ICC, IHC, WB</t>
         </is>
       </c>
     </row>
@@ -2057,12 +2065,12 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>IgG1</t>
+          <t>IgG (H+L)</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Alexa Fluor 488</t>
+          <t>Alexa Fluor Plus 647 (Goat, Invitrogen A32728)</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
@@ -2072,14 +2080,14 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Green</t>
+          <t>Far-Red</t>
         </is>
       </c>
       <c r="F10" s="6" t="n">
-        <v>490</v>
+        <v>650</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>525</v>
+        <v>665</v>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
@@ -2090,17 +2098,17 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Mouse</t>
+          <t>Rabbit</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>IgG1</t>
+          <t>IgG (H+L)</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Alexa Fluor 594</t>
+          <t>Alexa Fluor Plus 555 (Goat, Invitrogen A32732)</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -2114,10 +2122,10 @@
         </is>
       </c>
       <c r="F11" s="6" t="n">
-        <v>590</v>
+        <v>555</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>617</v>
+        <v>565</v>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
@@ -2128,17 +2136,17 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Mouse</t>
+          <t>Biotin</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>IgG1</t>
+          <t>Biotin</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Alexa Fluor 647</t>
+          <t>Alexa Fluor 488 (Streptavidin, Invitrogen S32354)</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -2148,434 +2156,16 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Far-Red</t>
+          <t>Green</t>
         </is>
       </c>
       <c r="F12" s="6" t="n">
-        <v>650</v>
+        <v>490</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>665</v>
+        <v>525</v>
       </c>
       <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>ICC, IHC, WB</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>Mouse</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>IgG2a</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Alexa Fluor 488</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>Fluorophore</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>Green</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="n">
-        <v>490</v>
-      </c>
-      <c r="G13" s="6" t="n">
-        <v>525</v>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>ICC, IHC, WB</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>Mouse</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>IgG2a</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Alexa Fluor 555</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>Fluorophore</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>Red</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="n">
-        <v>555</v>
-      </c>
-      <c r="G14" s="6" t="n">
-        <v>565</v>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>ICC, IHC, WB</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Mouse</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>IgG2a</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Alexa Fluor 647</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>Fluorophore</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t>Far-Red</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="n">
-        <v>650</v>
-      </c>
-      <c r="G15" s="6" t="n">
-        <v>665</v>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>ICC, IHC, WB</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Mouse</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>IgG2b</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Alexa Fluor 488</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>Fluorophore</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>Green</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="n">
-        <v>490</v>
-      </c>
-      <c r="G16" s="6" t="n">
-        <v>525</v>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>ICC, IHC, WB</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>Mouse</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>IgG2b</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Alexa Fluor 555</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>Fluorophore</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>Red</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="n">
-        <v>555</v>
-      </c>
-      <c r="G17" s="6" t="n">
-        <v>565</v>
-      </c>
-      <c r="H17" s="5" t="inlineStr">
-        <is>
-          <t>ICC, IHC, WB</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>Mouse</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>IgG2b</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Alexa Fluor 647</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>Fluorophore</t>
-        </is>
-      </c>
-      <c r="E18" s="6" t="inlineStr">
-        <is>
-          <t>Far-Red</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="n">
-        <v>650</v>
-      </c>
-      <c r="G18" s="6" t="n">
-        <v>665</v>
-      </c>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>ICC, IHC, WB</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>Mouse</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>IgM</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Alexa Fluor 488</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>Fluorophore</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>Green</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="n">
-        <v>490</v>
-      </c>
-      <c r="G19" s="6" t="n">
-        <v>525</v>
-      </c>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t>ICC, IHC, WB</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>Mouse</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>IgM</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Alexa Fluor 555</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>Fluorophore</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="inlineStr">
-        <is>
-          <t>Red</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="n">
-        <v>555</v>
-      </c>
-      <c r="G20" s="6" t="n">
-        <v>565</v>
-      </c>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t>ICC, IHC, WB</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>Mouse</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>IgM</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Alexa Fluor 647</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>Fluorophore</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>Far-Red</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="n">
-        <v>650</v>
-      </c>
-      <c r="G21" s="6" t="n">
-        <v>665</v>
-      </c>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>ICC, IHC, WB</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>Rat</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>IgG (H+L)</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Alexa Fluor 647</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>Fluorophore</t>
-        </is>
-      </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>Far-Red</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="n">
-        <v>650</v>
-      </c>
-      <c r="G22" s="6" t="n">
-        <v>665</v>
-      </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>ICC, IHC, WB</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>Chicken</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>IgY (H+L)</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>Alexa Fluor 647</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>Fluorophore</t>
-        </is>
-      </c>
-      <c r="E23" s="6" t="inlineStr">
-        <is>
-          <t>Far-Red</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="n">
-        <v>650</v>
-      </c>
-      <c r="G23" s="6" t="n">
-        <v>665</v>
-      </c>
-      <c r="H23" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
@@ -2592,11 +2182,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
@@ -2828,6 +2418,34 @@
       <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Streptavidin-AF488 (S32354)</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Biotinylated Targets</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>490</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>525</v>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Make combination cards independently scrollable, pin designer options and export bar, and remove upload/download buttons from top header
</commit_message>
<xml_diff>
--- a/data/SpectraPanel_Database_Populated.xlsx
+++ b/data/SpectraPanel_Database_Populated.xlsx
@@ -476,16 +476,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="85" customWidth="1" min="1" max="1"/>
+    <col width="95" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SpectraPanel v1.0 — Streamlined Database Template</t>
+          <t>SpectraPanel v1.0 — Laboratory Inventory Database Template</t>
         </is>
       </c>
     </row>
@@ -502,28 +502,28 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>1. This template is stripped down to strictly what is required for multiplex panel design.</t>
+          <t>1. Keep the column headers in row 1 unchanged across all sheets.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2. Keep the column headers in row 1 unchanged.</t>
+          <t>2. Enter your laboratory's antibody and reagent inventory into the respective sheets.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>3. Enter your lab's inventory across the respective sheets (Primaries, Secondaries, Direct_Dyes, Reporters).</t>
+          <t>3. Detection channels for Secondaries and Reporters are computed dynamically in SpectraPanel based on emission wavelengths.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>4. Save this workbook and click 'Upload Database' in SpectraPanel to load everything in one click.</t>
+          <t>4. Save this workbook and click 'Upload Database' in SpectraPanel to import all sheets at once.</t>
         </is>
       </c>
     </row>
@@ -533,49 +533,226 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Accepted Values &amp; Conventions:</t>
+          <t>Sheet Column Reference &amp; Conventions:</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>• applications: Comma-separated (e.g., 'ICC, IHC, WB' or 'ICC, IHC')</t>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>• Primaries Sheet:</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>• live_cell_compatible: 'Yes' or 'No'</t>
+          <t xml:space="preserve">    - target: Target protein or marker (e.g., 'Pax7', 'alpha-Tubulin')</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>• color: 'Blue', 'Green', 'Orange', 'Red', 'Far-Red', 'Near-IR'</t>
+          <t xml:space="preserve">    - clonality: 'Monoclonal', 'Polyclonal', or 'Recombinant Monoclonal'</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>• conjugate_type: 'Fluorophore' or 'HRP'</t>
+          <t xml:space="preserve">    - clone: Clone name or ID (e.g., 'DM1A', '5.8A', 'PAX7/497')</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>• conjugated_color: Leave blank if unconjugated; enter fluorophore color if directly conjugated.</t>
+          <t xml:space="preserve">    - host: Primary host species (e.g., 'Mouse', 'Rabbit')</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>• fixation_compatible: 'PFA', 'Methanol', or 'PFA, Methanol'</t>
+          <t xml:space="preserve">    - isotype: Primary isotype (e.g., 'IgG1', 'IgG2a', 'IgG2b', 'IgG', 'IgM')</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    - make: Manufacturer / Supplier (e.g., 'Invitrogen', 'Sigma-Aldrich', 'DSHB', 'CST')</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    - catalog: Product catalog number</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    - applications: Comma-separated validated applications (e.g., 'ICC, IHC, WB')</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    - conjugated_color: Leave blank for unconjugated; enter fluorophore color if directly conjugated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    - fixation_compatible: 'PFA', 'Methanol', or 'PFA, Methanol'</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    - live_cell_compatible: 'Yes' or 'No'</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    - comments: Lab notes, storage box, aliquot notes, etc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>• Secondaries Sheet:</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    - anti_host: Target species recognized by the secondary (e.g., 'Mouse', 'Rabbit', 'Chicken')</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    - anti_isotype: Specific isotype recognized (e.g., 'IgG (H+L)', 'IgM', 'IgG1')</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    - host: Host animal species that produced the secondary antibody (e.g., 'Goat', 'Donkey')</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    - conjugate: Fluorophore or enzyme name (e.g., 'Alexa Fluor 488', 'Alexa Fluor Plus 647', 'HRP')</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    - conjugate_type: 'Fluorophore' or 'HRP'</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    - color: Optical color group ('Green', 'Red', 'Far-Red')</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    - excitation_nm: Peak excitation wavelength in nm (e.g., 490, 650)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    - emission_nm: Peak emission wavelength in nm (e.g., 525, 665)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    - applications: 'ICC, IHC, WB'</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    - make: Manufacturer / Supplier (e.g., 'Invitrogen')</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    - catalogue: Secondary antibody catalog number</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    - comments: Box location, receipt date, or lot notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>• Direct Dyes Sheet:</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    - name, target_structure, color, excitation_nm, emission_nm, live_cell_compatible, make, catalogue</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>• Reporters Sheet:</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    - reporter_name, color, excitation_nm, emission_nm, recommended_fixation</t>
         </is>
       </c>
     </row>
@@ -590,16 +767,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="29" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="23" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="33" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -610,32 +792,57 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
+          <t>clonality</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>clone</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
           <t>host</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>isotype</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>make</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>catalog</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>applications</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>conjugated_color</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>fixation_compatible</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>live_cell_compatible</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>comments</t>
         </is>
       </c>
     </row>
@@ -647,30 +854,51 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>PAX7/497</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>IgG1</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>NeoBiotechnologies</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>5081-MSM1-P0</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr"/>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="I2" s="5" t="inlineStr"/>
+      <c r="J2" s="5" t="inlineStr">
         <is>
           <t>PFA, Methanol</t>
         </is>
       </c>
-      <c r="G2" s="6" t="inlineStr">
+      <c r="K2" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
+      <c r="L2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -680,30 +908,51 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>5.8A</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>IgG1</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>BD Pharmingen</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>554130</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr"/>
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>PFA</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="K3" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
+      <c r="L3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -713,28 +962,53 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
+          <t>Recombinant Monoclonal</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>HL1372</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
           <t>Rabbit</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>IgG</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Invitrogen</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>MA5-47019</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr"/>
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>PFA</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="K4" s="6" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>Recombinant rabbit monoclonal</t>
         </is>
       </c>
     </row>
@@ -746,28 +1020,53 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
+          <t>Recombinant Monoclonal</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>7H1L69</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
           <t>Rabbit</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>IgG</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Invitrogen</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>701914</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>ICC, WB</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr"/>
+      <c r="J5" s="5" t="inlineStr">
         <is>
           <t>PFA, Methanol</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="K5" s="6" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>Recombinant rabbit monoclonal</t>
         </is>
       </c>
     </row>
@@ -779,28 +1078,53 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>9D10</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>IgM</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>DSHB</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>9D10</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr"/>
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>PFA, Methanol</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="K6" s="6" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>Hybridoma bank clone</t>
         </is>
       </c>
     </row>
@@ -812,28 +1136,53 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>mAb 5B12.3</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>IgG2a</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>DSHB</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>mAb 5B12.3</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr"/>
+      <c r="J7" s="5" t="inlineStr">
         <is>
           <t>Methanol</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="K7" s="6" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>Hybridoma bank clone</t>
         </is>
       </c>
     </row>
@@ -845,28 +1194,53 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>mAb 3F2.3</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>IgG2a</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>DSHB</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>mAb 3F2.3</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr"/>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr"/>
+      <c r="J8" s="5" t="inlineStr">
         <is>
           <t>Methanol</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="K8" s="6" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Hybridoma bank clone</t>
         </is>
       </c>
     </row>
@@ -878,28 +1252,53 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>JLT12</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>IgG1</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>DSHB</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>JLT12</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>ICC, WB</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr"/>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="I9" s="5" t="inlineStr"/>
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>PFA</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="K9" s="6" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>Hybridoma bank clone</t>
         </is>
       </c>
     </row>
@@ -911,28 +1310,53 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>MF 20</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>IgG2b</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>DSHB</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>MF 20</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr"/>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr"/>
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>PFA, Methanol</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="K10" s="6" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>Pan-sarcomeric MHC</t>
         </is>
       </c>
     </row>
@@ -944,28 +1368,53 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>PAX7</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="C11" s="6" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>IgG1</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>DSHB</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>PAX7</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr"/>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="I11" s="5" t="inlineStr"/>
+      <c r="J11" s="5" t="inlineStr">
         <is>
           <t>PFA, Methanol</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="K11" s="6" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>Hybridoma bank clone</t>
         </is>
       </c>
     </row>
@@ -977,28 +1426,53 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>TI-4</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>IgG1</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>DSHB</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>TI-4</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr"/>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="I12" s="5" t="inlineStr"/>
+      <c r="J12" s="5" t="inlineStr">
         <is>
           <t>PFA, Methanol</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="K12" s="6" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>Cardiac &amp; skeletal Troponin I</t>
         </is>
       </c>
     </row>
@@ -1010,28 +1484,53 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>mMaC myomesin B4</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>IgG1</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>DSHB</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>mMaC myomesin B4</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr"/>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="I13" s="5" t="inlineStr"/>
+      <c r="J13" s="5" t="inlineStr">
         <is>
           <t>PFA, Methanol</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="K13" s="6" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>M-band marker</t>
         </is>
       </c>
     </row>
@@ -1043,30 +1542,51 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>GA1R</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>IgG1</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Invitrogen</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>MA5-15738</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr"/>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="I14" s="5" t="inlineStr"/>
+      <c r="J14" s="5" t="inlineStr">
         <is>
           <t>PFA, Methanol</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="K14" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
+      <c r="L14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -1076,30 +1596,51 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
+          <t>Polyclonal</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Polyclonal</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
           <t>Rabbit</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>IgG</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Proteintech</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>14948-1-AP</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr"/>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="I15" s="5" t="inlineStr"/>
+      <c r="J15" s="5" t="inlineStr">
         <is>
           <t>PFA, Methanol</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="K15" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
+      <c r="L15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -1109,28 +1650,53 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>636</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>IgG2b</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Santa Cruz</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>sc-7292</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr"/>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="I16" s="5" t="inlineStr"/>
+      <c r="J16" s="5" t="inlineStr">
         <is>
           <t>PFA, Methanol</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="K16" s="6" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>Nuclear envelope marker</t>
         </is>
       </c>
     </row>
@@ -1142,30 +1708,51 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>NX-38</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>IgG2a</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Sigma-Aldrich</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>SAB4200124</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
         <is>
           <t>ICC, WB</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr"/>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="I17" s="5" t="inlineStr"/>
+      <c r="J17" s="5" t="inlineStr">
         <is>
           <t>PFA, Methanol</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="K17" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
+      <c r="L17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1175,28 +1762,53 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>D18C11</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
           <t>Rabbit</t>
         </is>
       </c>
-      <c r="C18" s="6" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>IgG</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Cell Signaling Technology</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>8456</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E18" s="5" t="inlineStr"/>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="I18" s="5" t="inlineStr"/>
+      <c r="J18" s="5" t="inlineStr">
         <is>
           <t>PFA</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="K18" s="6" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>Rabbit monoclonal</t>
         </is>
       </c>
     </row>
@@ -1208,30 +1820,51 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>PAX7/497</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>IgG1</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>NeoBiotechnologies</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>5081-MSM1</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr"/>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="I19" s="5" t="inlineStr"/>
+      <c r="J19" s="5" t="inlineStr">
         <is>
           <t>PFA, Methanol</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="K19" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
+      <c r="L19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -1241,28 +1874,53 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>EA-53</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="C20" s="6" t="inlineStr">
+      <c r="E20" s="6" t="inlineStr">
         <is>
           <t>IgG1</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Sigma-Aldrich</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>A7811</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr"/>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="I20" s="5" t="inlineStr"/>
+      <c r="J20" s="5" t="inlineStr">
         <is>
           <t>PFA, Methanol</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="K20" s="6" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>Z-line marker</t>
         </is>
       </c>
     </row>
@@ -1274,30 +1932,51 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>G-11</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>IgG1</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Santa Cruz</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>sc-25327</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr"/>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="I21" s="5" t="inlineStr"/>
+      <c r="J21" s="5" t="inlineStr">
         <is>
           <t>PFA, Methanol</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr">
+      <c r="K21" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
+      <c r="L21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -1307,30 +1986,51 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>P4D1</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
+      <c r="E22" s="6" t="inlineStr">
         <is>
           <t>IgG1</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Enzo Life Sciences</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>BML-PW0930-0100</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E22" s="5" t="inlineStr"/>
-      <c r="F22" s="5" t="inlineStr">
+      <c r="I22" s="5" t="inlineStr"/>
+      <c r="J22" s="5" t="inlineStr">
         <is>
           <t>PFA, Methanol</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="K22" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
+      <c r="L22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -1340,30 +2040,51 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>VI-10</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="C23" s="6" t="inlineStr">
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t>IgM</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Invitrogen</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>MA1-10459</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr"/>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="I23" s="5" t="inlineStr"/>
+      <c r="J23" s="5" t="inlineStr">
         <is>
           <t>PFA, Methanol</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr">
+      <c r="K23" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
+      <c r="L23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -1373,30 +2094,51 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>DM1A</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
+      <c r="E24" s="6" t="inlineStr">
         <is>
           <t>IgG1</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Sigma-Aldrich</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>T9026</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr"/>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="I24" s="5" t="inlineStr"/>
+      <c r="J24" s="5" t="inlineStr">
         <is>
           <t>PFA, Methanol</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="K24" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
+      <c r="L24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -1406,30 +2148,51 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>DM1A</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>IgG1</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Invitrogen</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>62204</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr"/>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="I25" s="5" t="inlineStr"/>
+      <c r="J25" s="5" t="inlineStr">
         <is>
           <t>PFA, Methanol</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr">
+      <c r="K25" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
+      <c r="L25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -1439,28 +2202,53 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>D13E12</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
           <t>Rabbit</t>
         </is>
       </c>
-      <c r="C26" s="6" t="inlineStr">
+      <c r="E26" s="6" t="inlineStr">
         <is>
           <t>IgG</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Cell Signaling Technology</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>6487</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
         <is>
           <t>ICC, WB</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr"/>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="I26" s="5" t="inlineStr"/>
+      <c r="J26" s="5" t="inlineStr">
         <is>
           <t>PFA</t>
         </is>
       </c>
-      <c r="G26" s="6" t="inlineStr">
+      <c r="K26" s="6" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>Rabbit monoclonal</t>
         </is>
       </c>
     </row>
@@ -1472,30 +2260,51 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>5C5</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="C27" s="6" t="inlineStr">
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>IgM</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Santa Cruz</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>sc-58670</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr"/>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="I27" s="5" t="inlineStr"/>
+      <c r="J27" s="5" t="inlineStr">
         <is>
           <t>PFA, Methanol</t>
         </is>
       </c>
-      <c r="G27" s="6" t="inlineStr">
+      <c r="K27" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
+      <c r="L27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -1505,30 +2314,51 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>15G5A11/E2</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="C28" s="6" t="inlineStr">
+      <c r="E28" s="6" t="inlineStr">
         <is>
           <t>IgG1</t>
         </is>
       </c>
-      <c r="D28" s="5" t="inlineStr">
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Invitrogen</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>MA1-140</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
         <is>
           <t>ICC, WB</t>
         </is>
       </c>
-      <c r="E28" s="5" t="inlineStr"/>
-      <c r="F28" s="5" t="inlineStr">
+      <c r="I28" s="5" t="inlineStr"/>
+      <c r="J28" s="5" t="inlineStr">
         <is>
           <t>PFA, Methanol</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr">
+      <c r="K28" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
+      <c r="L28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -1538,30 +2368,51 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>AC-74</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="C29" s="6" t="inlineStr">
+      <c r="E29" s="6" t="inlineStr">
         <is>
           <t>IgG2a</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Sigma-Aldrich</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>A2228</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E29" s="5" t="inlineStr"/>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="I29" s="5" t="inlineStr"/>
+      <c r="J29" s="5" t="inlineStr">
         <is>
           <t>PFA, Methanol</t>
         </is>
       </c>
-      <c r="G29" s="6" t="inlineStr">
+      <c r="K29" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
+      <c r="L29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -1571,28 +2422,53 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
+          <t>Polyclonal</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Polyclonal</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
           <t>Rabbit</t>
         </is>
       </c>
-      <c r="C30" s="6" t="inlineStr">
+      <c r="E30" s="6" t="inlineStr">
         <is>
           <t>IgG</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Sigma-Aldrich</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>ABT264</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
         <is>
           <t>ICC, WB</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr"/>
-      <c r="F30" s="5" t="inlineStr">
+      <c r="I30" s="5" t="inlineStr"/>
+      <c r="J30" s="5" t="inlineStr">
         <is>
           <t>PFA, Methanol</t>
         </is>
       </c>
-      <c r="G30" s="6" t="inlineStr">
+      <c r="K30" s="6" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="L30" s="5" t="inlineStr">
+        <is>
+          <t>Arginylated beta-Actin</t>
         </is>
       </c>
     </row>
@@ -1604,30 +2480,51 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>2A3</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="C31" s="6" t="inlineStr">
+      <c r="E31" s="6" t="inlineStr">
         <is>
           <t>IgG2b</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Abcam</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>ab123034</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr"/>
-      <c r="F31" s="5" t="inlineStr">
+      <c r="I31" s="5" t="inlineStr"/>
+      <c r="J31" s="5" t="inlineStr">
         <is>
           <t>PFA, Methanol</t>
         </is>
       </c>
-      <c r="G31" s="6" t="inlineStr">
+      <c r="K31" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
+      <c r="L31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -1637,28 +2534,53 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>D18C11</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
           <t>Rabbit</t>
         </is>
       </c>
-      <c r="C32" s="6" t="inlineStr">
+      <c r="E32" s="6" t="inlineStr">
         <is>
           <t>IgG</t>
         </is>
       </c>
-      <c r="D32" s="5" t="inlineStr">
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Cell Signaling Technology</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>8456</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E32" s="5" t="inlineStr"/>
-      <c r="F32" s="5" t="inlineStr">
+      <c r="I32" s="5" t="inlineStr"/>
+      <c r="J32" s="5" t="inlineStr">
         <is>
           <t>PFA</t>
         </is>
       </c>
-      <c r="G32" s="6" t="inlineStr">
+      <c r="K32" s="6" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="L32" s="5" t="inlineStr">
+        <is>
+          <t>Rabbit monoclonal</t>
         </is>
       </c>
     </row>
@@ -1670,30 +2592,51 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
+          <t>Monoclonal</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>1A4</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
           <t>Mouse</t>
         </is>
       </c>
-      <c r="C33" s="6" t="inlineStr">
+      <c r="E33" s="6" t="inlineStr">
         <is>
           <t>IgG2a</t>
         </is>
       </c>
-      <c r="D33" s="5" t="inlineStr">
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Sigma-Aldrich</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>A2547</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
         </is>
       </c>
-      <c r="E33" s="5" t="inlineStr"/>
-      <c r="F33" s="5" t="inlineStr">
+      <c r="I33" s="5" t="inlineStr"/>
+      <c r="J33" s="5" t="inlineStr">
         <is>
           <t>PFA, Methanol</t>
         </is>
       </c>
-      <c r="G33" s="6" t="inlineStr">
+      <c r="K33" s="6" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
+      <c r="L33" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1706,17 +2649,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="53" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="33" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1732,32 +2679,52 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
+          <t>host</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
           <t>conjugate</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>conjugate_type</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>color</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>excitation_nm</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>emission_nm</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>applications</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>make</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>catalogue</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>comments</t>
         </is>
       </c>
     </row>
@@ -1772,22 +2739,42 @@
           <t>IgG (H+L)</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>HRP (Donkey, Invitrogen A15999)</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>Donkey</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>HRP</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr"/>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>HRP</t>
+        </is>
+      </c>
       <c r="F2" s="6" t="inlineStr"/>
       <c r="G2" s="6" t="inlineStr"/>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr"/>
+      <c r="I2" s="5" t="inlineStr">
         <is>
           <t>WB</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Invitrogen</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>A15999</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>Donkey anti-Goat HRP</t>
         </is>
       </c>
     </row>
@@ -1802,30 +2789,50 @@
           <t>IgM</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>Alexa Fluor 488 (Goat, Invitrogen A21042)</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Goat</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Alexa Fluor 488</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>Fluorophore</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
         <is>
           <t>Green</t>
         </is>
       </c>
-      <c r="F3" s="6" t="n">
+      <c r="G3" s="6" t="n">
         <v>490</v>
       </c>
-      <c r="G3" s="6" t="n">
+      <c r="H3" s="6" t="n">
         <v>525</v>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Invitrogen</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>A21042</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>Goat anti-Mouse IgM (µ chain)</t>
         </is>
       </c>
     </row>
@@ -1840,30 +2847,50 @@
           <t>IgG (H+L)</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Alexa Fluor 488 (Donkey, Invitrogen A21206)</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Donkey</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Alexa Fluor 488</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>Fluorophore</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Green</t>
         </is>
       </c>
-      <c r="F4" s="6" t="n">
+      <c r="G4" s="6" t="n">
         <v>490</v>
       </c>
-      <c r="G4" s="6" t="n">
+      <c r="H4" s="6" t="n">
         <v>525</v>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Invitrogen</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>A21206</t>
+        </is>
+      </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>Received Jan 2020</t>
         </is>
       </c>
     </row>
@@ -1878,30 +2905,50 @@
           <t>IgY (H+L)</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Alexa Fluor 633 (Goat, Invitrogen A21103)</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Goat</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Alexa Fluor 633</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>Fluorophore</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Far-Red</t>
         </is>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="G5" s="6" t="n">
         <v>632</v>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="H5" s="6" t="n">
         <v>647</v>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Invitrogen</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>A21103</t>
+        </is>
+      </c>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>Common 4 deg box</t>
         </is>
       </c>
     </row>
@@ -1916,30 +2963,50 @@
           <t>IgG (H+L)</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Alexa Fluor 647 (Goat, Invitrogen A21245)</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Goat</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Alexa Fluor 647</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Fluorophore</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Far-Red</t>
         </is>
       </c>
-      <c r="F6" s="6" t="n">
+      <c r="G6" s="6" t="n">
         <v>650</v>
       </c>
-      <c r="G6" s="6" t="n">
+      <c r="H6" s="6" t="n">
         <v>665</v>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Invitrogen</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>A21245</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>Goat anti-Rabbit IgG (H+L)</t>
         </is>
       </c>
     </row>
@@ -1954,30 +3021,50 @@
           <t>IgG (H+L)</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Alexa Fluor 647 (Goat, Invitrogen A21235)</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Goat</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Alexa Fluor 647</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>Fluorophore</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Far-Red</t>
         </is>
       </c>
-      <c r="F7" s="6" t="n">
+      <c r="G7" s="6" t="n">
         <v>650</v>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="H7" s="6" t="n">
         <v>665</v>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>Invitrogen</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>A21235</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>Goat anti-Mouse IgG (H+L)</t>
         </is>
       </c>
     </row>
@@ -1992,30 +3079,50 @@
           <t>IgG (H+L)</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Alexa Fluor 488 (Goat, Invitrogen A11001)</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Goat</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Alexa Fluor 488</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>Fluorophore</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Green</t>
         </is>
       </c>
-      <c r="F8" s="6" t="n">
+      <c r="G8" s="6" t="n">
         <v>490</v>
       </c>
-      <c r="G8" s="6" t="n">
+      <c r="H8" s="6" t="n">
         <v>525</v>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Invitrogen</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>A11001</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Goat anti-Mouse IgG (H+L)</t>
         </is>
       </c>
     </row>
@@ -2030,30 +3137,50 @@
           <t>IgG (H+L)</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Alexa Fluor Plus 647 (Goat, Invitrogen A32733)</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Goat</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Alexa Fluor Plus 647</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>Fluorophore</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>Far-Red</t>
         </is>
       </c>
-      <c r="F9" s="6" t="n">
+      <c r="G9" s="6" t="n">
         <v>650</v>
       </c>
-      <c r="G9" s="6" t="n">
+      <c r="H9" s="6" t="n">
         <v>665</v>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>Invitrogen</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>A32733</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>Alexa Fluor Plus 647</t>
         </is>
       </c>
     </row>
@@ -2068,30 +3195,50 @@
           <t>IgG (H+L)</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Alexa Fluor Plus 647 (Goat, Invitrogen A32728)</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Goat</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Alexa Fluor Plus 647</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>Fluorophore</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Far-Red</t>
         </is>
       </c>
-      <c r="F10" s="6" t="n">
+      <c r="G10" s="6" t="n">
         <v>650</v>
       </c>
-      <c r="G10" s="6" t="n">
+      <c r="H10" s="6" t="n">
         <v>665</v>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Invitrogen</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>A32728</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>Alexa Fluor Plus 647</t>
         </is>
       </c>
     </row>
@@ -2106,30 +3253,50 @@
           <t>IgG (H+L)</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Alexa Fluor Plus 555 (Goat, Invitrogen A32732)</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Goat</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Alexa Fluor Plus 555</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>Fluorophore</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
       </c>
-      <c r="F11" s="6" t="n">
+      <c r="G11" s="6" t="n">
         <v>555</v>
       </c>
-      <c r="G11" s="6" t="n">
+      <c r="H11" s="6" t="n">
         <v>565</v>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="I11" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>Invitrogen</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>A32732</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>Alexa Fluor Plus 555</t>
         </is>
       </c>
     </row>
@@ -2144,30 +3311,50 @@
           <t>Biotin</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Alexa Fluor 488 (Streptavidin, Invitrogen S32354)</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Streptavidin</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Alexa Fluor 488</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>Fluorophore</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Green</t>
         </is>
       </c>
-      <c r="F12" s="6" t="n">
+      <c r="G12" s="6" t="n">
         <v>490</v>
       </c>
-      <c r="G12" s="6" t="n">
+      <c r="H12" s="6" t="n">
         <v>525</v>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="I12" s="5" t="inlineStr">
         <is>
           <t>ICC, IHC, WB</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>Invitrogen</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>S32354</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>Streptavidin AF488 conjugate</t>
         </is>
       </c>
     </row>
@@ -2182,15 +3369,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
-    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2224,6 +3413,16 @@
           <t>live_cell_compatible</t>
         </is>
       </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>make</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>catalogue</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -2252,6 +3451,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Invitrogen</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>D1306</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -2280,6 +3489,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Invitrogen</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>H1399</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -2308,6 +3527,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Invitrogen</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>A12379</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -2336,6 +3565,16 @@
           <t>No</t>
         </is>
       </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Invitrogen</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>A12381</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -2364,6 +3603,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Spirochrome</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>CY-SC001</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -2392,6 +3641,16 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Invitrogen</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>M7512</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -2420,11 +3679,21 @@
           <t>Yes</t>
         </is>
       </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Invitrogen</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>W11261</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Streptavidin-AF488 (S32354)</t>
+          <t>Streptavidin-AF488</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
@@ -2446,6 +3715,16 @@
       <c r="F9" s="6" t="inlineStr">
         <is>
           <t>No</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Invitrogen</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>S32354</t>
         </is>
       </c>
     </row>

</xml_diff>